<commit_message>
Finance model: use shop thread's chosen domain and PO box costs
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K99p7wLhiS2HD3dTBbm83j
</commit_message>
<xml_diff>
--- a/moodius-aurelius/business/finance/moodius-finance-model.xlsx
+++ b/moodius-aurelius/business/finance/moodius-finance-model.xlsx
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="745">
   <si>
     <t xml:space="preserve">Moodius Aurelius: financial model</t>
   </si>
@@ -835,6 +835,12 @@
     <t xml:space="preserve">Put your starting budget here; the cash view shows if it ever goes below zero.</t>
   </si>
   <si>
+    <t xml:space="preserve">PO box postage deposit (one-off, refundable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i-support Post Forwarding deposit; paid in month 1 of the cash view.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Share of a month's sales paid out the next month</t>
   </si>
   <si>
@@ -895,13 +901,13 @@
     <t xml:space="preserve">Needs your OK</t>
   </si>
   <si>
-    <t xml:space="preserve">About £10 a year, shown per month. Paid upfront in the cash view.</t>
+    <t xml:space="preserve">About £8 a year at Cloudflare cost price (shop thread, 22 Oct), shown per month. Paid upfront in the cash view.</t>
   </si>
   <si>
     <t xml:space="preserve">PO box / virtual address</t>
   </si>
   <si>
-    <t xml:space="preserve">£5-15 a month, midpoint. Legally needed on the shop's legal pages and in marketing emails.</t>
+    <t xml:space="preserve">i-support Post Forwarding £13/mo (or £130/yr), picked by the shop thread 22 Oct; plus a £20 one-off postage deposit in the cash view. Legally needed on the legal pages and in marketing emails.</t>
   </si>
   <si>
     <t xml:space="preserve">VPS for comment agent + n8n</t>
@@ -1492,7 +1498,7 @@
     <t xml:space="preserve">  of which fixed costs paid this month £</t>
   </si>
   <si>
-    <t xml:space="preserve">Domain's year paid in M1.</t>
+    <t xml:space="preserve">Domain's year and the PO box deposit paid in M1.</t>
   </si>
   <si>
     <t xml:space="preserve">Closing cash £</t>
@@ -3041,15 +3047,15 @@
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">'Fixed costs'!$D$17</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'Fixed costs'!$D$17</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">'Fixed costs'!$D$17</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>13</v>
@@ -3061,15 +3067,15 @@
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">'Fixed costs'!$D$17*Inputs!$C$6</f>
-        <v>32.4583333333333</v>
+        <v>35.7166666666667</v>
       </c>
       <c r="C12" s="11" t="n">
         <f aca="false">'Fixed costs'!$D$17*Inputs!$C$6</f>
-        <v>32.4583333333333</v>
+        <v>35.7166666666667</v>
       </c>
       <c r="D12" s="11" t="n">
         <f aca="false">'Fixed costs'!$D$17*Inputs!$C$6</f>
-        <v>32.4583333333333</v>
+        <v>35.7166666666667</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>15</v>
@@ -3101,15 +3107,15 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">Scenarios!$B$29</f>
-        <v>2.77788792652169</v>
+        <v>3.05674650913273</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">Scenarios!$C$29</f>
-        <v>2.77788792652169</v>
+        <v>3.05674650913273</v>
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">Scenarios!$D$29</f>
-        <v>2.77788792652169</v>
+        <v>3.05674650913273</v>
       </c>
       <c r="E14" s="10"/>
     </row>
@@ -3139,15 +3145,15 @@
       </c>
       <c r="B16" s="13" t="n">
         <f aca="false">Scenarios!$B$28</f>
-        <v>163861.862035498</v>
+        <v>180311.152935595</v>
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">Scenarios!$C$28</f>
-        <v>39737.9066827361</v>
+        <v>43727.0007810544</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">Scenarios!$D$28</f>
-        <v>9265.47969872358</v>
+        <v>10195.5958892758</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>22</v>
@@ -3177,15 +3183,15 @@
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">Scenarios!$B$39</f>
-        <v>-83.0983740030783</v>
+        <v>-91.5983740030783</v>
       </c>
       <c r="C18" s="9" t="n">
         <f aca="false">Scenarios!$C$39</f>
-        <v>-66.6707027330783</v>
+        <v>-75.1707027330783</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">Scenarios!$D$39</f>
-        <v>102.202201753322</v>
+        <v>93.7022017533218</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>25</v>
@@ -3384,58 +3390,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">Journals!$B$6</f>
@@ -3457,7 +3463,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="H5" s="17" t="n">
         <v>3</v>
@@ -3475,15 +3481,15 @@
         <v>6</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">Inputs!$C$52</f>
@@ -3505,7 +3511,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="H6" s="17" t="n">
         <v>2</v>
@@ -3523,15 +3529,15 @@
         <v>12</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">Inputs!$C$70</f>
@@ -3553,7 +3559,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="H7" s="17" t="n">
         <v>3</v>
@@ -3571,15 +3577,15 @@
         <v>11</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">Merch!$B$6+Merch!$B$7</f>
@@ -3601,7 +3607,7 @@
         <v>2</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="H8" s="17" t="n">
         <v>3</v>
@@ -3619,15 +3625,15 @@
         <v>8</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">'Rate card'!$D$10</f>
@@ -3649,7 +3655,7 @@
         <v>3</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="H9" s="17" t="n">
         <v>1</v>
@@ -3667,15 +3673,15 @@
         <v>10</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">Inputs!$C$65</f>
@@ -3697,7 +3703,7 @@
         <v>3</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="H10" s="17" t="n">
         <v>15</v>
@@ -3715,15 +3721,15 @@
         <v>1</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">Inputs!$C$54</f>
@@ -3745,7 +3751,7 @@
         <v>3</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="H11" s="13" t="n">
         <f aca="false">1000*Inputs!$C$58</f>
@@ -3764,15 +3770,15 @@
         <v>4</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">Inputs!$C$64</f>
@@ -3794,7 +3800,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>3</v>
@@ -3812,15 +3818,15 @@
         <v>2</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">Inputs!$C$63</f>
@@ -3842,7 +3848,7 @@
         <v>5</v>
       </c>
       <c r="G13" s="38" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>4</v>
@@ -3860,10 +3866,10 @@
         <v>5</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3890,7 +3896,7 @@
         <v>4</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>15</v>
@@ -3908,10 +3914,10 @@
         <v>9</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3938,7 +3944,7 @@
         <v>5</v>
       </c>
       <c r="G15" s="38" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>3</v>
@@ -3956,15 +3962,15 @@
         <v>7</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Inputs!$C$68</f>
@@ -3986,7 +3992,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
@@ -4004,10 +4010,10 @@
         <v>3</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -4039,40 +4045,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">Inputs!$C$20</f>
@@ -4086,15 +4092,15 @@
         <v>Not yet</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">Inputs!$C$16</f>
@@ -4108,15 +4114,15 @@
         <v>Not yet</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">Inputs!$C$13</f>
@@ -4131,15 +4137,15 @@
         <v>Met</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="C8" s="23"/>
       <c r="D8" s="9" t="n">
@@ -4151,15 +4157,15 @@
         <v>No data</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">Inputs!$C$17</f>
@@ -4174,15 +4180,15 @@
         <v>Not yet</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">Inputs!$C$17</f>
@@ -4196,7 +4202,7 @@
         <v>Not yet</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4204,7 +4210,7 @@
         <v>100</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">Inputs!$C$19</f>
@@ -4218,15 +4224,15 @@
         <v>Not yet</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="C12" s="13" t="n">
         <f aca="false">Inputs!$C$9</f>
@@ -4240,15 +4246,15 @@
         <v>Not yet</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">Inputs!$C$12</f>
@@ -4262,15 +4268,15 @@
         <v>Not yet</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="C14" s="13" t="n">
         <f aca="false">Inputs!$C$12</f>
@@ -4284,15 +4290,15 @@
         <v>Not yet</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C15" s="13" t="n">
         <f aca="false">Inputs!$C$16+Inputs!$C$18</f>
@@ -4306,7 +4312,7 @@
         <v>Not yet</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4314,7 +4320,7 @@
         <v>98</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">Inputs!$C$18</f>
@@ -4328,15 +4334,15 @@
         <v>Not yet</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C17" s="13" t="n">
         <f aca="false">Inputs!$C$16+Inputs!$C$18</f>
@@ -4350,12 +4356,12 @@
         <v>Not yet</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B18" s="38" t="s">
         <v>206</v>
@@ -4372,15 +4378,15 @@
         <v>Not yet</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B19" s="38" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="17" t="n">
@@ -4391,7 +4397,7 @@
         <v>No data</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4433,133 +4439,133 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="39" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="D4" s="38" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="39" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="39" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="39" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="39" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="39" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="39" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
   </sheetData>
@@ -4590,7 +4596,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4598,181 +4604,181 @@
         <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="39" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="D4" s="40" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="39" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="D5" s="40" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="39" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="C6" s="38" t="s">
+        <v>690</v>
+      </c>
+      <c r="D6" s="40" t="s">
         <v>688</v>
-      </c>
-      <c r="D6" s="40" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="39" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="D7" s="40" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="39" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="39" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B10" s="38" t="s">
+        <v>702</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>703</v>
+      </c>
+      <c r="D10" s="40" t="s">
         <v>700</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>701</v>
-      </c>
-      <c r="D10" s="40" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="39" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="39" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="39" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="39" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="B14" s="38" t="s">
         <v>49</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="39" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="C15" s="38" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="D15" s="40" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
   </sheetData>
@@ -4801,95 +4807,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
     </row>
   </sheetData>
@@ -4909,7 +4915,7 @@
     <tabColor rgb="FFC9742E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -6086,14 +6092,14 @@
       <c r="B75" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="C75" s="18" t="n">
-        <v>0.25</v>
+      <c r="C75" s="20" t="n">
+        <v>20</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>67</v>
+        <v>109</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>221</v>
@@ -6103,17 +6109,34 @@
       <c r="B76" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="C76" s="19" t="n">
+      <c r="C76" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F76" s="10" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C77" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D76" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="E76" s="5" t="s">
+      <c r="D77" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="F76" s="10" t="s">
-        <v>224</v>
+      <c r="F77" s="10" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -6146,35 +6169,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>64</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>11</v>
@@ -6182,10 +6205,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C5" s="21" t="n">
         <v>20</v>
@@ -6202,74 +6225,74 @@
         <v>1</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6" s="24" t="n">
         <f aca="false">IF(B6="GBP",C6,C6/Inputs!$C$6)/12</f>
-        <v>0.833333333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="E6" s="25" t="n">
         <f aca="false">D6*Inputs!$C$6</f>
-        <v>0.958333333333333</v>
+        <v>0.766666666666667</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H6" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>238</v>
-      </c>
       <c r="C7" s="20" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D7" s="24" t="n">
         <f aca="false">IF(B7="GBP",C7,C7/Inputs!$C$6)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E7" s="25" t="n">
         <f aca="false">D7*Inputs!$C$6</f>
-        <v>11.5</v>
+        <v>14.95</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C8" s="21" t="n">
         <v>5</v>
@@ -6286,18 +6309,18 @@
         <v>0</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C9" s="21" t="n">
         <v>5</v>
@@ -6314,18 +6337,18 @@
         <v>0</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C10" s="20" t="n">
         <v>0</v>
@@ -6342,18 +6365,18 @@
         <v>1</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C11" s="20" t="n">
         <v>0</v>
@@ -6370,18 +6393,18 @@
         <v>1</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C12" s="20" t="n">
         <v>0</v>
@@ -6398,18 +6421,18 @@
         <v>1</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C13" s="20" t="n">
         <v>0</v>
@@ -6426,18 +6449,18 @@
         <v>1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C14" s="20" t="n">
         <v>0</v>
@@ -6454,16 +6477,16 @@
         <v>1</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="H14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C15" s="20" t="n">
         <v>0</v>
@@ -6480,41 +6503,41 @@
         <v>0</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D17" s="26" t="n">
         <f aca="false">SUMPRODUCT(D5:D15,F5:F15)</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="E17" s="27" t="n">
         <f aca="false">D17*Inputs!$C$6</f>
-        <v>32.4583333333333</v>
+        <v>35.7166666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D18" s="24" t="n">
         <f aca="false">SUM(D5:D15)</f>
-        <v>36.9202898550725</v>
+        <v>39.7536231884058</v>
       </c>
       <c r="E18" s="25" t="n">
         <f aca="false">D18*Inputs!$C$6</f>
-        <v>42.4583333333333</v>
+        <v>45.7166666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D19" s="24" t="n">
         <f aca="false">E19/Inputs!$C$6</f>
@@ -6526,15 +6549,15 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D20" s="24" t="n">
         <f aca="false">D19-D17</f>
-        <v>-6.48550724637681</v>
+        <v>-9.31884057971015</v>
       </c>
       <c r="E20" s="25" t="n">
         <f aca="false">E19-E17</f>
-        <v>-7.45833333333334</v>
+        <v>-10.7166666666667</v>
       </c>
     </row>
   </sheetData>
@@ -6569,58 +6592,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>0</v>
@@ -6664,12 +6687,12 @@
         <v>0</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>14</v>
@@ -6713,12 +6736,12 @@
         <v>10.77</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>6</v>
@@ -6762,12 +6785,12 @@
         <v>4.5</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>9</v>
@@ -6811,12 +6834,12 @@
         <v>6.85</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>29</v>
@@ -6860,12 +6883,12 @@
         <v>22.52</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B10" s="20" t="n">
         <v>15</v>
@@ -6909,12 +6932,12 @@
         <v>11.55</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B11" s="20" t="n">
         <v>19</v>
@@ -6958,12 +6981,12 @@
         <v>13.93</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B12" s="20" t="n">
         <v>22</v>
@@ -7007,12 +7030,12 @@
         <v>16.03</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B13" s="20" t="n">
         <v>34</v>
@@ -7056,17 +7079,17 @@
         <v>25.68</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Inputs!$C$70</f>
@@ -7075,7 +7098,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B17" s="24" t="n">
         <f aca="false">Inputs!$C$70*Inputs!$C$71-Inputs!$C$72</f>
@@ -7084,7 +7107,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">Inputs!$C$72</f>
@@ -7093,12 +7116,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B21" s="29" t="n">
         <f aca="false">SUMPRODUCT(--(ABS(F5:F13-L5:L13)&gt;0.011))</f>
@@ -7134,17 +7157,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
@@ -7153,16 +7176,16 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8" t="s">
@@ -7171,7 +7194,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>28</v>
@@ -7183,12 +7206,12 @@
         <v>28</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>3.95</v>
@@ -7200,12 +7223,12 @@
         <v>6.95</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B8" s="26" t="n">
         <f aca="false">B6+B7</f>
@@ -7223,7 +7246,7 @@
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B9" s="22" t="n">
         <v>12.95</v>
@@ -7235,12 +7258,12 @@
         <v>12.95</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B10" s="24" t="n">
         <f aca="false">B9*Inputs!$C$7</f>
@@ -7255,12 +7278,12 @@
         <v>9.7125</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="false">3.99*Inputs!$C$7</f>
@@ -7275,12 +7298,12 @@
         <v>2.9925</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B12" s="20" t="n">
         <v>0</v>
@@ -7292,12 +7315,12 @@
         <v>0</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B13" s="24" t="n">
         <f aca="false">Inputs!$C$43*Inputs!$C$7</f>
@@ -7315,7 +7338,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B14" s="24" t="n">
         <f aca="false">B8*Inputs!$C$44</f>
@@ -7330,12 +7353,12 @@
         <v>2.27175</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B15" s="24" t="n">
         <f aca="false">B8*Inputs!$C$45+Inputs!$C$46</f>
@@ -7350,12 +7373,12 @@
         <v>1.598</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B16" s="24" t="n">
         <f aca="false">(B13+B14+B15)*Inputs!$C$47</f>
@@ -7370,12 +7393,12 @@
         <v>0.80395</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B17" s="24" t="n">
         <f aca="false">B6*Inputs!$C$48</f>
@@ -7390,12 +7413,12 @@
         <v>1.4</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B18" s="26" t="n">
         <f aca="false">B10+B11+B12+B13+B14+B15+B16+B17</f>
@@ -7413,7 +7436,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B19" s="26" t="n">
         <f aca="false">B8-B18</f>
@@ -7431,7 +7454,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B20" s="28" t="n">
         <f aca="false">IF(B8=0,0,B19/B8)</f>
@@ -7449,7 +7472,7 @@
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B21" s="24" t="n">
         <f aca="false">B8-B10-B11-B12-(B8*Inputs!$C$24+Inputs!$C$27)-B17</f>
@@ -7464,12 +7487,12 @@
         <v>18.845075</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -7478,16 +7501,16 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8" t="s">
@@ -7496,7 +7519,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B25" s="20" t="n">
         <v>22</v>
@@ -7508,12 +7531,12 @@
         <v>22</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B26" s="20" t="n">
         <v>3.95</v>
@@ -7525,12 +7548,12 @@
         <v>6.95</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B27" s="26" t="n">
         <f aca="false">B25+B26</f>
@@ -7548,7 +7571,7 @@
     </row>
     <row r="28" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B28" s="22" t="n">
         <v>10.95</v>
@@ -7560,12 +7583,12 @@
         <v>10.95</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B29" s="24" t="n">
         <f aca="false">B28*Inputs!$C$7</f>
@@ -7580,12 +7603,12 @@
         <v>8.2125</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B30" s="20" t="n">
         <f aca="false">4.99</f>
@@ -7600,12 +7623,12 @@
         <v>3.7425</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B31" s="20" t="n">
         <v>0</v>
@@ -7617,12 +7640,12 @@
         <v>0</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B32" s="24" t="n">
         <f aca="false">Inputs!$C$43*Inputs!$C$7</f>
@@ -7640,7 +7663,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B33" s="24" t="n">
         <f aca="false">B27*Inputs!$C$44</f>
@@ -7655,12 +7678,12 @@
         <v>1.88175</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B34" s="24" t="n">
         <f aca="false">B27*Inputs!$C$45+Inputs!$C$46</f>
@@ -7675,12 +7698,12 @@
         <v>1.358</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B35" s="24" t="n">
         <f aca="false">(B32+B33+B34)*Inputs!$C$47</f>
@@ -7695,12 +7718,12 @@
         <v>0.67795</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B36" s="24" t="n">
         <f aca="false">B25*Inputs!$C$48</f>
@@ -7715,12 +7738,12 @@
         <v>1.1</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B37" s="26" t="n">
         <f aca="false">B29+B30+B31+B32+B33+B34+B35+B36</f>
@@ -7738,7 +7761,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B38" s="26" t="n">
         <f aca="false">B27-B37</f>
@@ -7756,7 +7779,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B39" s="28" t="n">
         <f aca="false">IF(B27=0,0,B38/B27)</f>
@@ -7774,7 +7797,7 @@
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B40" s="24" t="n">
         <f aca="false">B27-B29-B30-B31-(B27*Inputs!$C$24+Inputs!$C$27)-B36</f>
@@ -7789,12 +7812,12 @@
         <v>14.204075</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
@@ -7803,16 +7826,16 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E43" s="8"/>
       <c r="F43" s="8" t="s">
@@ -7821,7 +7844,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B44" s="20" t="n">
         <v>22</v>
@@ -7833,12 +7856,12 @@
         <v>22</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B45" s="20" t="n">
         <v>3.95</v>
@@ -7850,12 +7873,12 @@
         <v>6.95</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B46" s="26" t="n">
         <f aca="false">B44+B45</f>
@@ -7873,7 +7896,7 @@
     </row>
     <row r="47" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B47" s="22" t="n">
         <v>15</v>
@@ -7885,12 +7908,12 @@
         <v>15</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B48" s="24" t="n">
         <f aca="false">B47*Inputs!$C$7</f>
@@ -7905,12 +7928,12 @@
         <v>11.25</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B49" s="20" t="n">
         <f aca="false">5.99*Inputs!$C$7</f>
@@ -7925,12 +7948,12 @@
         <v>4.4925</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B50" s="20" t="n">
         <v>0</v>
@@ -7942,12 +7965,12 @@
         <v>0</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B51" s="24" t="n">
         <f aca="false">Inputs!$C$43*Inputs!$C$7</f>
@@ -7965,7 +7988,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B52" s="24" t="n">
         <f aca="false">B46*Inputs!$C$44</f>
@@ -7980,12 +8003,12 @@
         <v>1.88175</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B53" s="24" t="n">
         <f aca="false">B46*Inputs!$C$45+Inputs!$C$46</f>
@@ -8000,12 +8023,12 @@
         <v>1.358</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B54" s="24" t="n">
         <f aca="false">(B51+B52+B53)*Inputs!$C$47</f>
@@ -8020,12 +8043,12 @@
         <v>0.67795</v>
       </c>
       <c r="F54" s="10" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B55" s="24" t="n">
         <f aca="false">B44*Inputs!$C$48</f>
@@ -8040,12 +8063,12 @@
         <v>1.1</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B56" s="26" t="n">
         <f aca="false">B48+B49+B50+B51+B52+B53+B54+B55</f>
@@ -8063,7 +8086,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B57" s="26" t="n">
         <f aca="false">B46-B56</f>
@@ -8081,7 +8104,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B58" s="28" t="n">
         <f aca="false">IF(B46=0,0,B57/B46)</f>
@@ -8099,7 +8122,7 @@
     </row>
     <row r="59" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B59" s="24" t="n">
         <f aca="false">B46-B48-B49-B50-(B46*Inputs!$C$24+Inputs!$C$27)-B55</f>
@@ -8114,29 +8137,29 @@
         <v>10.416575</v>
       </c>
       <c r="F59" s="10" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B61" s="9" t="n">
         <f aca="false">Inputs!$C$49</f>
         <v>45</v>
       </c>
       <c r="F61" s="10" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B64" s="9" t="n">
         <f aca="false">Journals!$J$6</f>
@@ -8145,7 +8168,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B65" s="9" t="n">
         <f aca="false">Merch!$B$19</f>
@@ -8154,7 +8177,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B66" s="9" t="n">
         <f aca="false">Merch!$B$38</f>
@@ -8163,7 +8186,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B67" s="9" t="n">
         <f aca="false">Merch!$B$57</f>
@@ -8172,7 +8195,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="30" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B69" s="30"/>
       <c r="C69" s="30"/>
@@ -8226,17 +8249,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>8</v>
@@ -8248,12 +8271,12 @@
         <v>10</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B5" s="17" t="n">
         <v>30</v>
@@ -8265,12 +8288,12 @@
         <v>30</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">Inputs!$C$12</f>
@@ -8283,12 +8306,12 @@
         <v>1000</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B7" s="31" t="n">
         <v>2</v>
@@ -8300,12 +8323,12 @@
         <v>8</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B8" s="18" t="n">
         <v>0.2</v>
@@ -8317,12 +8340,12 @@
         <v>0.4</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B9" s="18" t="n">
         <v>0.01</v>
@@ -8334,12 +8357,12 @@
         <v>0.04</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>0.005</v>
@@ -8351,12 +8374,12 @@
         <v>0.02</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B11" s="31" t="n">
         <v>0.5</v>
@@ -8368,12 +8391,12 @@
         <v>2</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
@@ -8382,7 +8405,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B14" s="32" t="n">
         <f aca="false">B5*B6</f>
@@ -8399,7 +8422,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B15" s="33" t="n">
         <f aca="false">B14/1000*B7</f>
@@ -8416,7 +8439,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B16" s="33" t="n">
         <f aca="false">B15*B8</f>
@@ -8433,7 +8456,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B17" s="33" t="n">
         <f aca="false">B16*B9+B15*B10</f>
@@ -8450,7 +8473,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B18" s="24" t="n">
         <f aca="false">B17*Journals!$B$6</f>
@@ -8467,7 +8490,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B19" s="24" t="n">
         <f aca="false">B17*Journals!$J$6</f>
@@ -8484,7 +8507,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B20" s="24" t="n">
         <f aca="false">B14/1000*B11*Inputs!$C$53*Inputs!$C$52*Inputs!$C$51</f>
@@ -8501,7 +8524,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B21" s="24" t="n">
         <f aca="false">B19+B20</f>
@@ -8518,58 +8541,58 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B22" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$17</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$17</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="D22" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$17</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B23" s="26" t="n">
         <f aca="false">B21-B22</f>
-        <v>-27.5528762011594</v>
+        <v>-30.3862095344928</v>
       </c>
       <c r="C23" s="26" t="n">
         <f aca="false">C21-C22</f>
-        <v>-19.7013992811594</v>
+        <v>-22.5347326144928</v>
       </c>
       <c r="D23" s="26" t="n">
         <f aca="false">D21-D22</f>
-        <v>63.1617943188406</v>
+        <v>60.3284609855073</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B24" s="25" t="n">
         <f aca="false">B23*Inputs!$C$6</f>
-        <v>-31.6858076313333</v>
+        <v>-34.9441409646667</v>
       </c>
       <c r="C24" s="25" t="n">
         <f aca="false">C23*Inputs!$C$6</f>
-        <v>-22.6566091733333</v>
+        <v>-25.9149425066667</v>
       </c>
       <c r="D24" s="25" t="n">
         <f aca="false">D23*Inputs!$C$6</f>
-        <v>72.6360634666667</v>
+        <v>69.3777301333333</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B25" s="26" t="n">
         <f aca="false">IF(B14=0,0,(B18+B20)/B14*1000)</f>
@@ -8586,7 +8609,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B26" s="24" t="n">
         <f aca="false">IF(B14=0,0,B21/B14*1000)</f>
@@ -8603,7 +8626,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B27" s="24" t="n">
         <f aca="false">B9*Journals!$J$6</f>
@@ -8620,57 +8643,57 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">IF(B26=0,0,B22/B26*1000)</f>
-        <v>163861.862035498</v>
+        <v>180311.152935595</v>
       </c>
       <c r="C28" s="29" t="n">
         <f aca="false">IF(C26=0,0,C22/C26*1000)</f>
-        <v>39737.9066827361</v>
+        <v>43727.0007810544</v>
       </c>
       <c r="D28" s="29" t="n">
         <f aca="false">IF(D26=0,0,D22/D26*1000)</f>
-        <v>9265.47969872358</v>
+        <v>10195.5958892758</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B29" s="33" t="n">
         <f aca="false">IF(Journals!$J$6=0,0,B22/Journals!$J$6)</f>
-        <v>2.77788792652169</v>
+        <v>3.05674650913273</v>
       </c>
       <c r="C29" s="33" t="n">
         <f aca="false">IF(Journals!$J$6=0,0,C22/Journals!$J$6)</f>
-        <v>2.77788792652169</v>
+        <v>3.05674650913273</v>
       </c>
       <c r="D29" s="33" t="n">
         <f aca="false">IF(Journals!$J$6=0,0,D22/Journals!$J$6)</f>
-        <v>2.77788792652169</v>
+        <v>3.05674650913273</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B31" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>8</v>
@@ -8687,27 +8710,27 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B35" s="33" t="n">
-        <f aca="false">(IF(1&gt;=Inputs!$C$76,Inputs!$C$10+(B14-Inputs!$C$10)/3,0)+IF(2&gt;=Inputs!$C$76,Inputs!$C$10+(B14-Inputs!$C$10)*2/3,0)+IF(3&gt;=Inputs!$C$76,B14,0))*(B7/1000*(B8*B9+B10))</f>
+        <f aca="false">(IF(1&gt;=Inputs!$C$77,Inputs!$C$10+(B14-Inputs!$C$10)/3,0)+IF(2&gt;=Inputs!$C$77,Inputs!$C$10+(B14-Inputs!$C$10)*2/3,0)+IF(3&gt;=Inputs!$C$77,B14,0))*(B7/1000*(B8*B9+B10))</f>
         <v>0.128058</v>
       </c>
       <c r="C35" s="33" t="n">
-        <f aca="false">(IF(1&gt;=Inputs!$C$76,Inputs!$C$10+(C14-Inputs!$C$10)/3,0)+IF(2&gt;=Inputs!$C$76,Inputs!$C$10+(C14-Inputs!$C$10)*2/3,0)+IF(3&gt;=Inputs!$C$76,C14,0))*(C7/1000*(C8*C9+C10))</f>
+        <f aca="false">(IF(1&gt;=Inputs!$C$77,Inputs!$C$10+(C14-Inputs!$C$10)/3,0)+IF(2&gt;=Inputs!$C$77,Inputs!$C$10+(C14-Inputs!$C$10)*2/3,0)+IF(3&gt;=Inputs!$C$77,C14,0))*(C7/1000*(C8*C9+C10))</f>
         <v>1.622208</v>
       </c>
       <c r="D35" s="33" t="n">
-        <f aca="false">(IF(1&gt;=Inputs!$C$76,Inputs!$C$10+(D14-Inputs!$C$10)/3,0)+IF(2&gt;=Inputs!$C$76,Inputs!$C$10+(D14-Inputs!$C$10)*2/3,0)+IF(3&gt;=Inputs!$C$76,D14,0))*(D7/1000*(D8*D9+D10))</f>
+        <f aca="false">(IF(1&gt;=Inputs!$C$77,Inputs!$C$10+(D14-Inputs!$C$10)/3,0)+IF(2&gt;=Inputs!$C$77,Inputs!$C$10+(D14-Inputs!$C$10)*2/3,0)+IF(3&gt;=Inputs!$C$77,D14,0))*(D7/1000*(D8*D9+D10))</f>
         <v>17.667936</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B36" s="24" t="n">
         <f aca="false">B35*Journals!$B$6+(3*Inputs!$C$10+(B14-Inputs!$C$10)*2)/1000*B11*Inputs!$C$53*Inputs!$C$52*Inputs!$C$51</f>
@@ -8724,7 +8747,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B37" s="24" t="n">
         <f aca="false">B35*Journals!$J$6+(3*Inputs!$C$10+(B14-Inputs!$C$10)*2)/1000*B11*Inputs!$C$53*Inputs!$C$52*Inputs!$C$51</f>
@@ -8741,53 +8764,53 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B38" s="24" t="n">
         <f aca="false">3*'Fixed costs'!$D$17</f>
-        <v>84.6739130434783</v>
+        <v>93.1739130434783</v>
       </c>
       <c r="C38" s="24" t="n">
         <f aca="false">3*'Fixed costs'!$D$17</f>
-        <v>84.6739130434783</v>
+        <v>93.1739130434783</v>
       </c>
       <c r="D38" s="24" t="n">
         <f aca="false">3*'Fixed costs'!$D$17</f>
-        <v>84.6739130434783</v>
+        <v>93.1739130434783</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B39" s="26" t="n">
         <f aca="false">B37-B38</f>
-        <v>-83.0983740030783</v>
+        <v>-91.5983740030783</v>
       </c>
       <c r="C39" s="26" t="n">
         <f aca="false">C37-C38</f>
-        <v>-66.6707027330783</v>
+        <v>-75.1707027330783</v>
       </c>
       <c r="D39" s="26" t="n">
         <f aca="false">D37-D38</f>
-        <v>102.202201753322</v>
+        <v>93.7022017533218</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B40" s="25" t="n">
         <f aca="false">B39*Inputs!$C$6</f>
-        <v>-95.56313010354</v>
+        <v>-105.33813010354</v>
       </c>
       <c r="C40" s="25" t="n">
         <f aca="false">C39*Inputs!$C$6</f>
-        <v>-76.67130814304</v>
+        <v>-86.44630814304</v>
       </c>
       <c r="D40" s="25" t="n">
         <f aca="false">D39*Inputs!$C$6</f>
-        <v>117.53253201632</v>
+        <v>107.75753201632</v>
       </c>
     </row>
   </sheetData>
@@ -8818,17 +8841,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B3" s="34" t="n">
         <v>2</v>
@@ -8836,19 +8859,19 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>11</v>
@@ -8856,21 +8879,21 @@
     </row>
     <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B7" s="32" t="n">
         <v>1</v>
@@ -8885,27 +8908,27 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B8" s="32" t="n">
-        <f aca="false">IF(B7&gt;=Inputs!$C$76,1,0)</f>
+        <f aca="false">IF(B7&gt;=Inputs!$C$77,1,0)</f>
         <v>1</v>
       </c>
       <c r="C8" s="32" t="n">
-        <f aca="false">IF(C7&gt;=Inputs!$C$76,1,0)</f>
+        <f aca="false">IF(C7&gt;=Inputs!$C$77,1,0)</f>
         <v>1</v>
       </c>
       <c r="D8" s="32" t="n">
-        <f aca="false">IF(D7&gt;=Inputs!$C$76,1,0)</f>
+        <f aca="false">IF(D7&gt;=Inputs!$C$77,1,0)</f>
         <v>1</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B9" s="32" t="n">
         <f aca="false">Inputs!$C$10+(INDEX(Scenarios!$B$14:$D$14,'90-day P&amp;L'!$B$3)-Inputs!$C$10)*B7/3</f>
@@ -8924,12 +8947,12 @@
         <v>25347</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B10" s="33" t="n">
         <f aca="false">B9/1000*INDEX(Scenarios!$B$7:$D$7,'90-day P&amp;L'!$B$3)</f>
@@ -8951,7 +8974,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B11" s="33" t="n">
         <f aca="false">B10*INDEX(Scenarios!$B$8:$D$8,'90-day P&amp;L'!$B$3)</f>
@@ -8973,7 +8996,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B12" s="33" t="n">
         <f aca="false">(B11*INDEX(Scenarios!$B$9:$D$9,'90-day P&amp;L'!$B$3)+B10*INDEX(Scenarios!$B$10:$D$10,'90-day P&amp;L'!$B$3))*B8</f>
@@ -8995,7 +9018,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B13" s="33" t="n">
         <f aca="false">B12+0</f>
@@ -9017,7 +9040,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B14" s="33" t="n">
         <f aca="false">IF(0&gt;=Inputs!$C$33,B12*0.3,0)</f>
@@ -9036,12 +9059,12 @@
         <v>0</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
@@ -9051,7 +9074,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B16" s="24" t="n">
         <f aca="false">B12*Journals!$B$6</f>
@@ -9073,7 +9096,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B17" s="24" t="n">
         <f aca="false">B14*Journals!$B$9</f>
@@ -9095,7 +9118,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B18" s="24" t="n">
         <f aca="false">B9/1000*INDEX(Scenarios!$B$11:$D$11,'90-day P&amp;L'!$B$3)*Inputs!$C$53*Inputs!$C$52*Inputs!$C$51</f>
@@ -9117,7 +9140,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B19" s="24" t="n">
         <f aca="false">0</f>
@@ -9136,12 +9159,12 @@
         <v>0</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B20" s="24" t="n">
         <f aca="false">0</f>
@@ -9160,12 +9183,12 @@
         <v>0</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B21" s="26" t="n">
         <f aca="false">SUM(B16:B20)</f>
@@ -9187,7 +9210,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -9197,7 +9220,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B23" s="24" t="n">
         <f aca="false">(B16+B17)*(1-1/(1+Inputs!$C$22))</f>
@@ -9216,12 +9239,12 @@
         <v>3.785152</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B24" s="24" t="n">
         <f aca="false">(B16+B17)/(1+Inputs!$C$22)-(B12*(Journals!$J$6+Journals!$B$6*Inputs!$C$29)+B14*(Journals!$J$9+Journals!$B$9*Inputs!$C$29))</f>
@@ -9240,12 +9263,12 @@
         <v>1.7620423296</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B25" s="24" t="n">
         <f aca="false">(B16+B17)*Inputs!$C$29</f>
@@ -9267,7 +9290,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B26" s="24" t="n">
         <f aca="false">0</f>
@@ -9286,12 +9309,12 @@
         <v>0</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B27" s="26" t="n">
         <f aca="false">B21-B23-B24-B25-B26</f>
@@ -9313,7 +9336,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -9323,7 +9346,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B29" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$5*'Fixed costs'!$F$5</f>
@@ -9345,31 +9368,31 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B30" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$17-B29</f>
-        <v>10.8333333333333</v>
+        <v>13.6666666666667</v>
       </c>
       <c r="C30" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$17-C29</f>
-        <v>10.8333333333333</v>
+        <v>13.6666666666667</v>
       </c>
       <c r="D30" s="24" t="n">
         <f aca="false">'Fixed costs'!$D$17-D29</f>
-        <v>10.8333333333333</v>
+        <v>13.6666666666667</v>
       </c>
       <c r="E30" s="26" t="n">
         <f aca="false">SUM(B30:D30)</f>
-        <v>32.5</v>
+        <v>41</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B31" s="20" t="n">
         <v>0</v>
@@ -9385,78 +9408,78 @@
         <v>0</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B32" s="24" t="n">
         <f aca="false">B29+B30+B31</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="C32" s="24" t="n">
         <f aca="false">C29+C30+C31</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="D32" s="24" t="n">
         <f aca="false">D29+D30+D31</f>
-        <v>28.2246376811594</v>
+        <v>31.0579710144928</v>
       </c>
       <c r="E32" s="26" t="n">
         <f aca="false">SUM(B32:D32)</f>
-        <v>84.6739130434783</v>
+        <v>93.1739130434783</v>
       </c>
       <c r="F32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B33" s="26" t="n">
         <f aca="false">B27-B32</f>
-        <v>-24.7457358742261</v>
+        <v>-27.5790692075594</v>
       </c>
       <c r="C33" s="26" t="n">
         <f aca="false">C27-C32</f>
-        <v>-22.2235675776928</v>
+        <v>-25.0569009110261</v>
       </c>
       <c r="D33" s="26" t="n">
         <f aca="false">D27-D32</f>
-        <v>-19.7013992811594</v>
+        <v>-22.5347326144928</v>
       </c>
       <c r="E33" s="26" t="n">
         <f aca="false">SUM(B33:D33)</f>
-        <v>-66.6707027330783</v>
+        <v>-75.1707027330783</v>
       </c>
       <c r="F33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B34" s="25" t="n">
         <f aca="false">B33*Inputs!$C$6</f>
-        <v>-28.45759625536</v>
+        <v>-31.7159295886933</v>
       </c>
       <c r="C34" s="25" t="n">
         <f aca="false">C33*Inputs!$C$6</f>
-        <v>-25.5571027143467</v>
+        <v>-28.81543604768</v>
       </c>
       <c r="D34" s="25" t="n">
         <f aca="false">D33*Inputs!$C$6</f>
-        <v>-22.6566091733333</v>
+        <v>-25.9149425066667</v>
       </c>
       <c r="E34" s="27" t="n">
         <f aca="false">SUM(B34:D34)</f>
-        <v>-76.67130814304</v>
+        <v>-86.44630814304</v>
       </c>
       <c r="F34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -9466,7 +9489,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B36" s="24" t="n">
         <f aca="false">Inputs!$C$74</f>
@@ -9474,30 +9497,30 @@
       </c>
       <c r="C36" s="24" t="n">
         <f aca="false">B40</f>
-        <v>-34.7821279926261</v>
+        <v>-55.7821279926261</v>
       </c>
       <c r="D36" s="24" t="n">
         <f aca="false">C40</f>
-        <v>-56.8029043111188</v>
+        <v>-80.8029043111189</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B37" s="24" t="n">
-        <f aca="false">(B27+B26)*(1-Inputs!$C$75)+0*Inputs!$C$75</f>
+        <f aca="false">(B27+B26)*(1-Inputs!$C$76)+0*Inputs!$C$76</f>
         <v>2.6091763552</v>
       </c>
       <c r="C37" s="24" t="n">
-        <f aca="false">(C27+C26)*(1-Inputs!$C$75)+(B27+B26)*Inputs!$C$75</f>
+        <f aca="false">(C27+C26)*(1-Inputs!$C$76)+(B27+B26)*Inputs!$C$76</f>
         <v>5.37052802933333</v>
       </c>
       <c r="D37" s="24" t="n">
-        <f aca="false">(D27+D26)*(1-Inputs!$C$75)+(C27+C26)*Inputs!$C$75</f>
+        <f aca="false">(D27+D26)*(1-Inputs!$C$76)+(C27+C26)*Inputs!$C$76</f>
         <v>7.89269632586667</v>
       </c>
       <c r="E37" s="26" t="n">
@@ -9508,82 +9531,82 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B38" s="24" t="n">
         <f aca="false">B32-B30+B39</f>
-        <v>37.3913043478261</v>
+        <v>58.3913043478261</v>
       </c>
       <c r="C38" s="24" t="n">
         <f aca="false">C32-C30+C39</f>
-        <v>27.3913043478261</v>
+        <v>30.3913043478261</v>
       </c>
       <c r="D38" s="24" t="n">
         <f aca="false">D32-D30+D39</f>
-        <v>27.3913043478261</v>
+        <v>30.3913043478261</v>
       </c>
       <c r="E38" s="26" t="n">
         <f aca="false">SUM(B38:D38)</f>
-        <v>92.1739130434783</v>
+        <v>119.173913043478</v>
       </c>
       <c r="F38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B39" s="24" t="n">
-        <f aca="false">B30-'Fixed costs'!$D$6*'Fixed costs'!$F$6+IF(B7=1,'Fixed costs'!$C$6*'Fixed costs'!$F$6,0)</f>
-        <v>20</v>
+        <f aca="false">B30-'Fixed costs'!$D$6*'Fixed costs'!$F$6+IF(B7=1,'Fixed costs'!$C$6*'Fixed costs'!$F$6+Inputs!$C$75,0)</f>
+        <v>41</v>
       </c>
       <c r="C39" s="24" t="n">
-        <f aca="false">C30-'Fixed costs'!$D$6*'Fixed costs'!$F$6+IF(C7=1,'Fixed costs'!$C$6*'Fixed costs'!$F$6,0)</f>
-        <v>10</v>
+        <f aca="false">C30-'Fixed costs'!$D$6*'Fixed costs'!$F$6+IF(C7=1,'Fixed costs'!$C$6*'Fixed costs'!$F$6+Inputs!$C$75,0)</f>
+        <v>13</v>
       </c>
       <c r="D39" s="24" t="n">
-        <f aca="false">D30-'Fixed costs'!$D$6*'Fixed costs'!$F$6+IF(D7=1,'Fixed costs'!$C$6*'Fixed costs'!$F$6,0)</f>
-        <v>10</v>
+        <f aca="false">D30-'Fixed costs'!$D$6*'Fixed costs'!$F$6+IF(D7=1,'Fixed costs'!$C$6*'Fixed costs'!$F$6+Inputs!$C$75,0)</f>
+        <v>13</v>
       </c>
       <c r="E39" s="26" t="n">
         <f aca="false">SUM(B39:D39)</f>
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B40" s="26" t="n">
         <f aca="false">B36+B37-B38</f>
-        <v>-34.7821279926261</v>
+        <v>-55.7821279926261</v>
       </c>
       <c r="C40" s="26" t="n">
         <f aca="false">C36+C37-C38</f>
-        <v>-56.8029043111188</v>
+        <v>-80.8029043111189</v>
       </c>
       <c r="D40" s="26" t="n">
         <f aca="false">D36+D37-D38</f>
-        <v>-76.3015123330783</v>
+        <v>-103.301512333078</v>
       </c>
       <c r="E40" s="26" t="n">
         <f aca="false">D40</f>
-        <v>-76.3015123330783</v>
+        <v>-103.301512333078</v>
       </c>
       <c r="F40" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B42" s="26" t="n">
         <f aca="false">MIN(B40:D40)</f>
-        <v>-76.3015123330783</v>
+        <v>-103.301512333078</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -9619,26 +9642,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>11</v>
@@ -9646,7 +9669,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B5" s="24" t="n">
         <f aca="false">Inputs!$C$35/Inputs!$C$6</f>
@@ -9661,12 +9684,12 @@
         <v>30.4347826086957</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B6" s="24" t="n">
         <f aca="false">Inputs!$C$37*Inputs!$C$7</f>
@@ -9681,12 +9704,12 @@
         <v>0.3</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B7" s="32" t="n">
         <f aca="false">B5/B6</f>
@@ -9704,7 +9727,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B8" s="32" t="n">
         <f aca="false">B5/(Inputs!$C$39*Inputs!$C$7)*1000</f>
@@ -9719,12 +9742,12 @@
         <v>10144.9275362319</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">Scenarios!$C$8</f>
@@ -9739,12 +9762,12 @@
         <v>0.3</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B10" s="33" t="n">
         <f aca="false">B7*B9</f>
@@ -9762,7 +9785,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B11" s="26" t="n">
         <f aca="false">IF(B10=0,0,B5/B10)</f>
@@ -9780,7 +9803,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B12" s="33" t="n">
         <f aca="false">B10*Scenarios!$C$9+B7*Scenarios!$C$10</f>
@@ -9795,12 +9818,12 @@
         <v>1.6231884057971</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B13" s="26" t="n">
         <f aca="false">IF(B12=0,0,B5/B12)</f>
@@ -9818,7 +9841,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B14" s="32" t="n">
         <f aca="false">B5/Inputs!$C$41</f>
@@ -9833,12 +9856,12 @@
         <v>101.449275362319</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B15" s="24" t="n">
         <f aca="false">IF(B14=0,0,B5/B14)</f>
@@ -9856,7 +9879,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B16" s="24" t="n">
         <f aca="false">B12*Journals!$J$6</f>
@@ -9874,7 +9897,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B17" s="36" t="n">
         <f aca="false">IF(B5=0,0,B16/B5)</f>
@@ -9889,12 +9912,12 @@
         <v>0.541891555555556</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -9903,7 +9926,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">Journals!$J$6</f>
@@ -9912,19 +9935,19 @@
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">Scenarios!$C$27</f>
         <v>0.203209333333333</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -9933,52 +9956,52 @@
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B24" s="23"/>
       <c r="E24" s="10" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B27" s="19"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B28" s="19"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B29" s="19"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B30" s="19"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B31" s="26" t="str">
         <f aca="false">IF(N(B27)=0,"",B24/B27)</f>
@@ -9987,7 +10010,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B32" s="26" t="str">
         <f aca="false">IF(N(B28)=0,"",B24/B28)</f>
@@ -9996,7 +10019,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B33" s="26" t="str">
         <f aca="false">IF(N(B29)=0,"",B24/B29)</f>
@@ -10005,7 +10028,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B34" s="26" t="str">
         <f aca="false">IF(N(B30)=0,"",B24/B30)</f>
@@ -10014,7 +10037,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B35" s="26" t="str">
         <f aca="false">IF(N(B25)=0,"",B24/B25*1000)</f>
@@ -10048,12 +10071,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10061,10 +10084,10 @@
         <v>33</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="s">
@@ -10073,7 +10096,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">Inputs!$C$12</f>
@@ -10083,12 +10106,12 @@
         <v>1000</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">Inputs!$C$9</f>
@@ -10100,7 +10123,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B7" s="37" t="n">
         <f aca="false">Inputs!$C$59</f>
@@ -10111,29 +10134,29 @@
         <v>15</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B10" s="24" t="n">
         <f aca="false">$B$5/1000*$B$7*Inputs!$C$7*1</f>
@@ -10148,13 +10171,13 @@
         <v>37.5</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="F10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B11" s="24" t="n">
         <f aca="false">$B$5/1000*$B$7*Inputs!$C$7*0.8</f>
@@ -10169,13 +10192,13 @@
         <v>30</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B12" s="24" t="n">
         <f aca="false">$B$5/1000*$B$7*Inputs!$C$7*0.5</f>
@@ -10190,13 +10213,13 @@
         <v>18.75</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B13" s="24" t="n">
         <f aca="false">$B$5/1000*$B$7*Inputs!$C$7*0.3</f>
@@ -10211,13 +10234,13 @@
         <v>11.25</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B14" s="24" t="n">
         <f aca="false">Inputs!$C$18*0.45/1000*25</f>
@@ -10232,13 +10255,13 @@
         <v>11.25</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B15" s="24" t="n">
         <f aca="false">$B$5/1000*$B$7*Inputs!$C$7*0.3</f>
@@ -10253,13 +10276,13 @@
         <v>11.25</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B16" s="24" t="n">
         <f aca="false">$B$5/1000*$B$7*Inputs!$C$7*0.25</f>
@@ -10274,132 +10297,132 @@
         <v>9.375</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="F16" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B18" s="3" t="str">
         <f aca="false">IF(AND(Inputs!$C$9&gt;=1000,Inputs!$C$12&gt;=1000),"Yes","Not yet")</f>
         <v>Not yet</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>520</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>518</v>
-      </c>
       <c r="E22" s="10" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>525</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>523</v>
-      </c>
       <c r="E24" s="10" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
   </sheetData>

</xml_diff>